<commit_message>
Add test data in providers file
</commit_message>
<xml_diff>
--- a/sfa.Tl.Marketing.Communication.DataLoad/Provider Data/Full Provider Data 2020 - 2021 (campaign site).xlsx
+++ b/sfa.Tl.Marketing.Communication.DataLoad/Provider Data/Full Provider Data 2020 - 2021 (campaign site).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\esfa\tl-marketing-and-communication\sfa.Tl.Marketing.Communication.DataLoad\Provider Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C60C83B-DD99-41D6-B895-30BCF28F8244}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF056FC3-1F66-4DD4-B927-8757DF400308}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4785" yWindow="2520" windowWidth="32790" windowHeight="16215" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13710" yWindow="2445" windowWidth="21435" windowHeight="17910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Provider Data 2020 - 2021" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8563" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8733" uniqueCount="603">
   <si>
     <t>Provider Name</t>
   </si>
@@ -1808,13 +1808,37 @@
   </si>
   <si>
     <t>Bristol</t>
+  </si>
+  <si>
+    <t>ESFA Test</t>
+  </si>
+  <si>
+    <t>CV1 2WT</t>
+  </si>
+  <si>
+    <t>Coventry</t>
+  </si>
+  <si>
+    <t>https://www.gov.uk/government/organisations/education-and-skills-funding-agency</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CV1 2NP</t>
+  </si>
+  <si>
+    <t>No courses for bug TLWP-1284</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CV1 2NL</t>
+  </si>
+  <si>
+    <t>No years for bug TLWP-1284</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1845,6 +1869,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1867,12 +1903,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2191,7 +2229,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:P605"/>
+  <dimension ref="A1:P617"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="44.28515625" customWidth="1"/>
@@ -30915,6 +30953,584 @@
       </c>
       <c r="P605" s="3" t="s">
         <v>579</v>
+      </c>
+    </row>
+    <row r="606" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A606" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B606" s="2"/>
+      <c r="C606" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D606" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E606" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O606" s="2">
+        <v>2020</v>
+      </c>
+      <c r="P606" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="607" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A607" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B607" s="2"/>
+      <c r="C607" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D607" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F607" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N607" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O607" s="2">
+        <v>2021</v>
+      </c>
+      <c r="P607" s="5" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="608" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A608" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B608" s="2"/>
+      <c r="C608" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D608" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G608" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N608" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O608" s="2">
+        <v>2022</v>
+      </c>
+      <c r="P608" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="609" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A609" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B609" s="2"/>
+      <c r="C609" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D609" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H609" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N609" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O609" s="2">
+        <v>2023</v>
+      </c>
+      <c r="P609" s="5" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="610" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A610" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B610" s="2"/>
+      <c r="C610" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D610" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I610" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N610" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O610" s="2">
+        <v>2021</v>
+      </c>
+      <c r="P610" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="611" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A611" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B611" s="2"/>
+      <c r="C611" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D611" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J611" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N611" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O611" s="2">
+        <v>2021</v>
+      </c>
+      <c r="P611" s="5" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="612" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A612" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B612" s="2"/>
+      <c r="C612" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D612" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K612" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N612" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O612" s="2">
+        <v>2022</v>
+      </c>
+      <c r="P612" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="613" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A613" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B613" s="2"/>
+      <c r="C613" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D613" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L613" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N613" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O613" s="2">
+        <v>2022</v>
+      </c>
+      <c r="P613" s="5" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="614" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A614" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B614" s="2"/>
+      <c r="C614" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D614" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M614" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="N614" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O614" s="2">
+        <v>2021</v>
+      </c>
+      <c r="P614" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="615" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A615" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B615" s="2"/>
+      <c r="C615" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D615" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M615" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N615" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="O615" s="2">
+        <v>2022</v>
+      </c>
+      <c r="P615" s="5" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="616" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A616" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B616" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="C616" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="D616" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N616" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O616" s="2">
+        <v>2021</v>
+      </c>
+      <c r="P616" s="5" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="617" spans="1:16" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A617" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B617" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="C617" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="D617" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N617" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O617" s="2"/>
+      <c r="P617" s="5" t="s">
+        <v>598</v>
       </c>
     </row>
   </sheetData>
@@ -31491,8 +32107,20 @@
     <hyperlink ref="P334" r:id="rId569" tooltip="Follow link" xr:uid="{3B62BD27-3557-49A5-8467-AB6348B3255E}"/>
     <hyperlink ref="P335" r:id="rId570" tooltip="Follow link" xr:uid="{82FA72EE-BB93-4D0E-82CA-51C739C648EC}"/>
     <hyperlink ref="P8" r:id="rId571" xr:uid="{3C7F5A7E-7811-430B-9E1E-12E9E13388CC}"/>
+    <hyperlink ref="P606" r:id="rId572" xr:uid="{DD541136-E40B-4BFD-8D2C-0A90E03B29AC}"/>
+    <hyperlink ref="P607" r:id="rId573" xr:uid="{919E6CC9-348D-42B2-A08E-E778F0DCD43A}"/>
+    <hyperlink ref="P608" r:id="rId574" xr:uid="{E781D1A8-BF19-4638-AEBB-0BDFF2A74BE9}"/>
+    <hyperlink ref="P609" r:id="rId575" xr:uid="{9A5669E6-8C43-4B61-A167-E772514EEA58}"/>
+    <hyperlink ref="P610" r:id="rId576" xr:uid="{944985E4-15C2-406B-8CDE-887A3E704674}"/>
+    <hyperlink ref="P611" r:id="rId577" xr:uid="{42778FA3-8AE1-4F3E-A0DE-9069F2DB5E68}"/>
+    <hyperlink ref="P612" r:id="rId578" xr:uid="{BB776BDE-2BDE-4E7B-988B-242461453606}"/>
+    <hyperlink ref="P613" r:id="rId579" xr:uid="{10403666-DA4E-45C5-880E-688AFC395836}"/>
+    <hyperlink ref="P614" r:id="rId580" xr:uid="{1DED6C2B-B628-4C0F-9900-F619F2F99D3A}"/>
+    <hyperlink ref="P615" r:id="rId581" xr:uid="{E6B74A01-028B-4263-A162-D19179B7AA88}"/>
+    <hyperlink ref="P616" r:id="rId582" xr:uid="{22AD1FD6-F54D-45D3-B872-C0F13AC91477}"/>
+    <hyperlink ref="P617" r:id="rId583" xr:uid="{7CDDE556-0D0A-43E8-8F22-3A6BCF55B12D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId572"/>
+  <pageSetup orientation="portrait" r:id="rId584"/>
 </worksheet>
 </file>
</xml_diff>